<commit_message>
Exemplo e testes cobrem casos de produção: desconto com totais, NF igual à AF, adiantamento sem NF, e-mail só com anexo
</commit_message>
<xml_diff>
--- a/modelo/Controle_Notas_exemplo.xlsx
+++ b/modelo/Controle_Notas_exemplo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Notas recebidas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Emails" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Revisao" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Guia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas recebidas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisao" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,13 +89,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -173,8 +173,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNotas" displayName="tbNotas" ref="A12:R20" headerRowCount="1">
-  <autoFilter ref="A12:R20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbNotas" displayName="tbNotas" ref="A12:R23" headerRowCount="1">
+  <autoFilter ref="A12:R23"/>
   <tableColumns count="18">
     <tableColumn id="1" name="NF"/>
     <tableColumn id="2" name="Empresa"/>
@@ -200,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbEmails" displayName="tbEmails" ref="A1:M4" headerRowCount="1">
-  <autoFilter ref="A1:M4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbEmails" displayName="tbEmails" ref="A1:M8" headerRowCount="1">
+  <autoFilter ref="A1:M8"/>
   <tableColumns count="13">
     <tableColumn id="1" name="ID_Email"/>
     <tableColumn id="2" name="Message_ID"/>
@@ -222,8 +222,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbRevisao" displayName="tbRevisao" ref="A1:F5" headerRowCount="1">
-  <autoFilter ref="A1:F5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tbRevisao" displayName="tbRevisao" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
   <tableColumns count="6">
     <tableColumn id="1" name="ID_Revisao"/>
     <tableColumn id="2" name="ID_Email"/>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:R20"/>
+  <dimension ref="A2:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -684,564 +684,765 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BETAVIARIA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Montagens Exemplo Ltda</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>5620</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Adiantamento — sem NF</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>46332.32291666667</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Não localizado nesta base</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Solicitação de adiantamento, não nota fiscal. Empresa: BETAVIARIA
+Solicitamos adiantamento conforme proposta.
+AF: 5620
+ | TEXTO1 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6|V13|TEXTO1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>BETAVIARIA|NOME:MONTAGENS EXEMPLO LTDA|NF:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>5530</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ALFAMETAL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Usinagem Fictícia Ltda</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2210</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>5530</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Envio informado</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>46332.25694444445</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Não localizado nesta base</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["2210","Usinagem Fictícia Ltda","5530","5530","20/11/2026"] | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5|V13|T1L2</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>ALFAMETAL|FOR:2210|NF:5530</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8120</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ALFAMETAL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Gases Modelo Ltda</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Desconto informado</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>46331.47222222222</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Não localizado nesta base</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["Gases Modelo Ltda","8120","1.500,00","150,00","1.350,00"] | Vencimento não informado | Instruções comunicadas: Bom dia, segue desconto negociado. FORNECEDOR NF VALOR NOTA FISCAL DIFERENÇA VALOR LÍQUIDO Gases Modelo Ltda 8120 1.500,00 150,00 1.350,00 TOTAL 1.500,00 150,00 1.350,00 Favor pagar o valor líquido. | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>1350</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4|V13|T1L2</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>ALFAMETAL|NOME:GASES MODELO LTDA|NF:8120</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>ALFAMETAL</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Fornecedor Exemplo Ltda</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>1020</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>5501</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F16" s="9" t="n">
         <v>46336</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Envio informado</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H16" s="10" t="n">
         <v>46331.38541666667</v>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>Aguardando conferência</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Possível duplicidade - conferir</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Dados de origem: ["ALFAMETAL","1020","Fornecedor Exemplo Ltda","1001","5501","10/11/2026"] | ENC/RES aceito; data de recebimento é a desta mensagem, não do envio original. | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
-        </is>
-      </c>
-      <c r="L13" s="8" t="n"/>
-      <c r="M13" s="8" t="n"/>
-      <c r="N13" s="8" t="n"/>
-      <c r="O13" s="8" t="n"/>
-      <c r="P13" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3|V13|T1L2</t>
-        </is>
-      </c>
-      <c r="R13" s="5" t="inlineStr">
-        <is>
-          <t>ALFAMETAL|FOR:1020|NF:1001</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>48213</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>ALFAMETAL</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Comercial Modelo ME</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>1187</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>5507</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>46338</v>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Envio informado</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>46331.38541666667</v>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Aguardando conferência</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>Possível duplicidade - conferir</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>Dados de origem: ["ALFAMETAL","1187","Comercial Modelo ME","48213","5507","12/11/2026"] | ENC/RES aceito; data de recebimento é a desta mensagem, não do envio original. | T1L3 | Referência de e-mail; documento fiscal não verificado.</t>
-        </is>
-      </c>
-      <c r="L14" s="8" t="n"/>
-      <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="n"/>
-      <c r="P14" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3</t>
-        </is>
-      </c>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3|V13|T1L3</t>
-        </is>
-      </c>
-      <c r="R14" s="5" t="inlineStr">
-        <is>
-          <t>ALFAMETAL|FOR:1187|NF:48213</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>2002/2003</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>BETAVIARIA</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Transportes Fictícios SA</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>3040</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>5502</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>46341</v>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Envio informado</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>46331.38541666667</v>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Aguardando conferência</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Possível duplicidade - conferir</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Dados de origem: ["BETAVIARIA","3040","Transportes Fictícios SA","2002/2003","5502","15/11/2026"] | ENC/RES aceito; data de recebimento é a desta mensagem, não do envio original. | T1L4 | Referência de e-mail; documento fiscal não verificado.</t>
-        </is>
-      </c>
-      <c r="L15" s="8" t="n"/>
-      <c r="M15" s="8" t="n"/>
-      <c r="N15" s="8" t="n"/>
-      <c r="O15" s="8" t="n"/>
-      <c r="P15" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3</t>
-        </is>
-      </c>
-      <c r="Q15" s="5" t="inlineStr">
-        <is>
-          <t>msg-exemplo-3|V13|T1L4</t>
-        </is>
-      </c>
-      <c r="R15" s="5" t="inlineStr">
-        <is>
-          <t>BETAVIARIA|FOR:3040|NF:2002/2003</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>777</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BETAVIARIA</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Serviços Demonstração Ltda</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>5610</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n">
-        <v>46357</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Envio informado</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>46330.56944444445</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Aguardando conferência</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Não localizado nesta base</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Dados de origem: ["Serviços Demonstração Ltda","777","5610","01/12/2026"] | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
         </is>
       </c>
       <c r="L16" s="11" t="n"/>
       <c r="M16" s="11" t="n"/>
       <c r="N16" s="11" t="n"/>
       <c r="O16" s="11" t="n"/>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>msg-exemplo-2</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>msg-exemplo-2|V13|T1L2</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>BETAVIARIA|NOME:SERVICOS DEMONSTRACAO LTDA|NF:777</t>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3|V13|T1L2</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>ALFAMETAL|FOR:1020|NF:1001</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>3315</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>BETAVIARIA</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Peças Exemplo Eireli</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>5611</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>48213</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>ALFAMETAL</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Comercial Modelo ME</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1187</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>5507</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>46338</v>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Envio informado</t>
         </is>
       </c>
       <c r="H17" s="10" t="n">
-        <v>46330.56944444445</v>
-      </c>
-      <c r="I17" t="inlineStr">
+        <v>46331.38541666667</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Aguardando conferência</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Não localizado nesta base</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Dados de origem: ["Peças Exemplo Eireli","3315","5611",""] | Vencimento não informado | T1L3 | Referência de e-mail; documento fiscal não verificado.</t>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Possível duplicidade - conferir</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["ALFAMETAL","1187","Comercial Modelo ME","48213","5507","12/11/2026"] | ENC/RES aceito; data de recebimento é a desta mensagem, não do envio original. | T1L3 | Referência de e-mail; documento fiscal não verificado.</t>
         </is>
       </c>
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
       <c r="N17" s="11" t="n"/>
       <c r="O17" s="11" t="n"/>
-      <c r="P17" t="inlineStr">
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3|V13|T1L3</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>ALFAMETAL|FOR:1187|NF:48213</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>2002/2003</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>BETAVIARIA</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Transportes Fictícios SA</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>3040</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>5502</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>46341</v>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Envio informado</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>46331.38541666667</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Possível duplicidade - conferir</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["BETAVIARIA","3040","Transportes Fictícios SA","2002/2003","5502","15/11/2026"] | ENC/RES aceito; data de recebimento é a desta mensagem, não do envio original. | T1L4 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="11" t="n"/>
+      <c r="O18" s="11" t="n"/>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-3|V13|T1L4</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t>BETAVIARIA|FOR:3040|NF:2002/2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>BETAVIARIA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Serviços Demonstração Ltda</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>5610</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>46357</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Envio informado</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>46330.56944444445</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Não localizado nesta base</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["Serviços Demonstração Ltda","777","5610","01/12/2026"] | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="7" t="n"/>
+      <c r="O19" s="7" t="n"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t>msg-exemplo-2</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>msg-exemplo-2|V13|T1L2</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>BETAVIARIA|NOME:SERVICOS DEMONSTRACAO LTDA|NF:777</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3315</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BETAVIARIA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Peças Exemplo Eireli</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>5611</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Envio informado</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>46330.56944444445</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Aguardando conferência</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Não localizado nesta base</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Dados de origem: ["Peças Exemplo Eireli","3315","5611",""] | Vencimento não informado | T1L3 | Referência de e-mail; documento fiscal não verificado.</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
+      <c r="O20" s="7" t="n"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>msg-exemplo-2</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>msg-exemplo-2|V13|T1L3</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>BETAVIARIA|NOME:PECAS EXEMPLO EIRELI|NF:3315</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>ALFAMETAL</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Fornecedor Exemplo Ltda</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>1020</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>5501</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F21" s="9" t="n">
         <v>46336</v>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Envio informado</t>
         </is>
       </c>
-      <c r="H18" s="7" t="n">
+      <c r="H21" s="10" t="n">
         <v>46329.42013888889</v>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Aguardando conferência</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>Não localizado nesta base</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>Dados de origem: ["ALFAMETAL","1020","Fornecedor Exemplo Ltda","1001","5501","10/11/2026"] | T1L2 | Referência de e-mail; documento fiscal não verificado.</t>
         </is>
       </c>
-      <c r="L18" s="8" t="n"/>
-      <c r="M18" s="8" t="n"/>
-      <c r="N18" s="8" t="n"/>
-      <c r="O18" s="8" t="n"/>
-      <c r="P18" s="5" t="inlineStr">
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1</t>
         </is>
       </c>
-      <c r="Q18" s="5" t="inlineStr">
+      <c r="Q21" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1|V13|T1L2</t>
         </is>
       </c>
-      <c r="R18" s="5" t="inlineStr">
+      <c r="R21" s="8" t="inlineStr">
         <is>
           <t>ALFAMETAL|FOR:1020|NF:1001</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>48213</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>ALFAMETAL</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Comercial Modelo ME</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>1187</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>5507</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F22" s="9" t="n">
         <v>46338</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>Envio informado</t>
         </is>
       </c>
-      <c r="H19" s="7" t="n">
+      <c r="H22" s="10" t="n">
         <v>46329.42013888889</v>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>Aguardando conferência</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Não localizado nesta base</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>Dados de origem: ["ALFAMETAL","1187","Comercial Modelo ME","48213","5507","12/11/2026"] | T1L3 | Referência de e-mail; documento fiscal não verificado.</t>
         </is>
       </c>
-      <c r="L19" s="8" t="n"/>
-      <c r="M19" s="8" t="n"/>
-      <c r="N19" s="8" t="n"/>
-      <c r="O19" s="8" t="n"/>
-      <c r="P19" s="5" t="inlineStr">
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
+      <c r="N22" s="11" t="n"/>
+      <c r="O22" s="11" t="n"/>
+      <c r="P22" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1</t>
         </is>
       </c>
-      <c r="Q19" s="5" t="inlineStr">
+      <c r="Q22" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1|V13|T1L3</t>
         </is>
       </c>
-      <c r="R19" s="5" t="inlineStr">
+      <c r="R22" s="8" t="inlineStr">
         <is>
           <t>ALFAMETAL|FOR:1187|NF:48213</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>2002/2003</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>BETAVIARIA</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Transportes Fictícios SA</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>3040</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>5502</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F23" s="9" t="n">
         <v>46341</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Envio informado</t>
         </is>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H23" s="10" t="n">
         <v>46329.42013888889</v>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Aguardando conferência</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>Não localizado nesta base</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
         <is>
           <t>Dados de origem: ["BETAVIARIA","3040","Transportes Fictícios SA","2002/2003","5502","15/11/2026"] | T1L4 | Referência de e-mail; documento fiscal não verificado.</t>
         </is>
       </c>
-      <c r="L20" s="8" t="n"/>
-      <c r="M20" s="8" t="n"/>
-      <c r="N20" s="8" t="n"/>
-      <c r="O20" s="8" t="n"/>
-      <c r="P20" s="5" t="inlineStr">
+      <c r="L23" s="11" t="n"/>
+      <c r="M23" s="11" t="n"/>
+      <c r="N23" s="11" t="n"/>
+      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1</t>
         </is>
       </c>
-      <c r="Q20" s="5" t="inlineStr">
+      <c r="Q23" s="8" t="inlineStr">
         <is>
           <t>msg-exemplo-1|V13|T1L4</t>
         </is>
       </c>
-      <c r="R20" s="5" t="inlineStr">
+      <c r="R23" s="8" t="inlineStr">
         <is>
           <t>BETAVIARIA|FOR:3040|NF:2002/2003</t>
         </is>
@@ -1261,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1357,7 +1558,7 @@
           <t>msg-exemplo-1</t>
         </is>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="6" t="n">
         <v>46329.42013888889</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -1435,7 +1636,7 @@
           <t>msg-exemplo-2</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="6" t="n">
         <v>46330.56944444445</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -1498,7 +1699,7 @@
           <t>msg-exemplo-3</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="6" t="n">
         <v>46331.38541666667</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -1565,6 +1766,245 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>46331.47222222222</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-11-05T14:20:00Z</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>compras@exemplo.com.br</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>DESCONTO: GASES MODELO X ALFAMETAL</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Com revisão</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Não informado pelo conector</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>[LEITOR_V13]
+Bom dia, segue desconto negociado.
+  FORNECEDOR
+NF
+VALOR NOTA FISCAL
+DIFERENÇA
+VALOR LÍQUIDO
+  Gases Modelo Ltda
+8120
+1.500,00
+150,00
+1.350,00
+  TOTAL
+1.500,00
+150,00
+1.350,00
+Favor pagar o valor líquido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46332.25694444445</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-11-06T09:10:00Z</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>compras@exemplo.com.br</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ENVIO DE NOTA FISCAL</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Com revisão</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Não informado pelo conector</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>[LEITOR_V13]
+Empresa: ALFAMETAL
+  FOR
+FORNECEDOR
+NF
+AF
+VENCIMENTO
+  2210
+Usinagem Fictícia Ltda
+5530
+5530
+20/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>46332.32291666667</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-11-06T10:45:00Z</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>compras@exemplo.com.br</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PAGAMENTO - Montagens Exemplo Ltda</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Com revisão</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Não informado pelo conector</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>[LEITOR_V13]
+Empresa: BETAVIARIA
+Solicitamos adiantamento conforme proposta.
+AF: 5620
+Atenciosamente,
+Compras</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-7</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>46332.52083333333</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-11-06T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>compras@exemplo.com.br</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>NF Peças Exemplo</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Com revisão</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Não informado pelo conector</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>[LEITOR_V13]
+Boa tarde, segue nota em anexo.
+Atenciosamente,
+Compras</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1579,7 +2019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1745,6 +2185,156 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4|V13P1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8120</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Campos incompletos / conferir</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>T1L2: Vencimento não informado. Linha preservada. ["Gases Modelo Ltda","8120","1.500,00","150,00","1.350,00"]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4|V13P2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>msg-exemplo-4</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>8120</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Validar desconto/ajuste</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>T1L2: valores e instruções transcritos, não autorizam pagamento. Conferir mensagem original.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5|V13P1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>msg-exemplo-5</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5530</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NF igual à AF</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>T1L2: números iguais preservados; não se concluiu que há erro.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6|V13P1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>msg-exemplo-6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Adiantamento sem NF</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Comunicação preservada fora dos totais de NF. Conferir o pedido e documentos; não confirma pagamento.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>msg-exemplo-7|V13P1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>msg-exemplo-7</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Formato não reconhecido</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mensagem preservada, sem extração segura. Não lê anexos/PDF/XML/imagens nem adivinha números e datas sem rótulos.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>

</xml_diff>